<commit_message>
Cap nhat thong tin TTCS_N1 mentor lich Sprint 1-4 va lien ket Jira da xac nhan
</commit_message>
<xml_diff>
--- a/theo-template/Danh_sach_can_bo_sung.xlsx
+++ b/theo-template/Danh_sach_can_bo_sung.xlsx
@@ -15,8 +15,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$G$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Thong tin nhom'!$A$1:$B$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SP thuc te'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Thong tin nhom'!$A$1:$B$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SP thuc te'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Git va dong gop'!$A$1:$L$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Ca nhan'!$A$1:$M$11</definedName>
   </definedNames>
@@ -528,10 +528,14 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Cần xác nhận</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+          <t>Đã cung cấp</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>TTCS_N1; mentor Triệu Quang Dũng; Đại học CNTT &amp; Truyền thông Thái Nguyên / CNTT / CNTT K23G; CodeGym.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="64" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -551,7 +555,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Ngày bắt đầu/kết thúc thực tập; ngày báo cáo; lịch Sprint 0–4</t>
+          <t>Ngày bắt đầu/kết thúc thực tập; ngày báo cáo; lịch Sprint 1–4</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -561,10 +565,14 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Chưa có</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
+          <t>Đã cung cấp</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Thực tập 23/09–26/10/2026; báo cáo 21/10/2026; S1 23–29/09; S2 30/09–06/10; S3 07–13/10; S4 14–20/10.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -627,10 +635,14 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Chưa có</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
+          <t>Đã có URL board; vẫn cần screenshot</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://ictu-team-k8abz7ih.atlassian.net/jira/software/projects/N1/boards/3/backlog</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="64" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -660,10 +672,14 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Đã có bản 18/10; cần bản mới nếu cập nhật</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>Có URL và export 18/10; cần export mới nếu cập nhật</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://ictu-team-k8abz7ih.atlassian.net/jira/software/projects/N1/boards/3/backlog</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -787,7 +803,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Cần khoảng thời gian/nhánh/phạm vi. Loại node_modules, tệp sinh tự động, ZIP khi tính dòng code.</t>
+          <t>Cần khoảng thời gian/nhánh/phạm vi. Loại node_modules, tệp sinh tự động, ZIP khi tính dòng code. Kỳ đã xác nhận: từ 23/09 đến thời điểm báo cáo 21/10/2026; không thống kê ngày sau đó.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1018,7 +1034,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Tổng cả nhóm phải 100%. Mentor xác nhận đúng số liệu cuối.</t>
+          <t>Tổng cả nhóm phải 100%. Mentor xác nhận đúng số liệu cuối. Mentor đã có tên Triệu Quang Dũng; chưa có xác nhận tỷ lệ.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1178,20 +1194,24 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận làm Phần B cho 10 thành viên hay chỉ Triệu Quang Dũng</t>
+          <t>Phần B cho cả 10 thành viên</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Bản hiện tại chuẩn bị đủ khung cho 10 người, ba slide/người; có thể rút lại khi bạn xác nhận.</t>
+          <t>Đã được người dùng xác nhận, giữ ba slide/người theo template.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Đang chờ trả lời</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
+          <t>Đã xác nhận</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Đã xác nhận: cả 10 thành viên, ba slide/người.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G22"/>
@@ -1205,7 +1225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1230,7 +1250,11 @@
           <t>Tên dự án chính thức</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise CRM — Hệ thống quản lý khách hàng</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1238,7 +1262,11 @@
           <t>Tên nhóm chính thức</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr"/>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>TTCS_N1</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1246,7 +1274,11 @@
           <t>Mentor</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Triệu Quang Dũng</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1254,7 +1286,11 @@
           <t>Đơn vị / phòng ban</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>CodeGym</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1262,7 +1298,11 @@
           <t>Trường</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Đại học CNTT &amp; Truyền thông Thái Nguyên</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1270,7 +1310,11 @@
           <t>Ngành</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>CNTT</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1278,7 +1322,11 @@
           <t>Lớp</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CNTT K23G</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1286,7 +1334,11 @@
           <t>Bắt đầu thực tập</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1294,7 +1346,11 @@
           <t>Kết thúc thực tập</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -1302,52 +1358,76 @@
           <t>Ngày báo cáo</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Sprint 0: từ / đến</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr"/>
+          <t>Sprint 1: từ / đến</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>23/09–29/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Sprint 1: từ / đến</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr"/>
+          <t>Sprint 2: từ / đến</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>30/09–06/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Sprint 2: từ / đến</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr"/>
+          <t>Sprint 3: từ / đến</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>07/10–13/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Sprint 3: từ / đến</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr"/>
+          <t>Sprint 4: từ / đến</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>14/10–20/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Sprint 4: từ / đến</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
+          <t>Độ dài sprint</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>1 tuần / 7 ngày</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Độ dài sprint</t>
+          <t>Lịch họp mentor</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr"/>
@@ -1355,7 +1435,7 @@
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lịch họp mentor</t>
+          <t>Kênh chat / thiết kế</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
@@ -1363,15 +1443,19 @@
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Kênh chat / thiết kế</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr"/>
+          <t>URL Jira board</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://ictu-team-k8abz7ih.atlassian.net/jira/software/projects/N1/boards/3/backlog</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>URL Jira board</t>
+          <t>URL deploy</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr"/>
@@ -1379,7 +1463,7 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>URL deploy</t>
+          <t>URL video demo</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr"/>
@@ -1387,7 +1471,7 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>URL video demo</t>
+          <t>Thứ tự người trình bày</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr"/>
@@ -1395,21 +1479,17 @@
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Thứ tự người trình bày</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
           <t>Phạm vi cá nhân: 10 người hay chỉ Leader</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Cả 10 thành viên</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B24"/>
+  <autoFilter ref="A1:B23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1420,7 +1500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1428,6 +1508,8 @@
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1456,6 +1538,16 @@
           <t>Nguồn / URL / ngày chụp</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Từ ngày</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Đến ngày</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1469,6 +1561,16 @@
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1482,6 +1584,16 @@
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
       <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1495,6 +1607,16 @@
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1508,9 +1630,19 @@
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
       <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:G5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>